<commit_message>
Table S2: store CI limits with two decimals; Table S3: add the SI-layout picture
The csv of Table S2 stored the Wilson limits with one decimal, so re-rounding them half-even could change a displayed value
(7/41: 8.53 -> 9, but 8.5 -> 8). Two decimals avoid this; the displayed table is unchanged. make_TableS3.py now also renders
TableS3_quality_by_model.png in the layout of the SI table (context-only block added).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/6_supplementary_figures/TableS2_generation_rate/TableS2_generation_rates.xlsx
+++ b/6_supplementary_figures/TableS2_generation_rate/TableS2_generation_rates.xlsx
@@ -645,7 +645,7 @@
         <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G2" t="n">
         <v>100</v>
@@ -672,7 +672,7 @@
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G3" t="n">
         <v>100</v>
@@ -699,7 +699,7 @@
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G4" t="n">
         <v>100</v>
@@ -726,7 +726,7 @@
         <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G5" t="n">
         <v>100</v>
@@ -750,13 +750,13 @@
         <v>41</v>
       </c>
       <c r="E6" t="n">
-        <v>17.1</v>
+        <v>17.07</v>
       </c>
       <c r="F6" t="n">
-        <v>8.5</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>31.3</v>
+        <v>31.26</v>
       </c>
     </row>
     <row r="7">
@@ -780,7 +780,7 @@
         <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G7" t="n">
         <v>100</v>
@@ -807,7 +807,7 @@
         <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G8" t="n">
         <v>100</v>
@@ -834,7 +834,7 @@
         <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G9" t="n">
         <v>100</v>
@@ -858,10 +858,10 @@
         <v>9</v>
       </c>
       <c r="E10" t="n">
-        <v>11.1</v>
+        <v>11.11</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="G10" t="n">
         <v>43.5</v>
@@ -885,13 +885,13 @@
         <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>44.4</v>
+        <v>44.44</v>
       </c>
       <c r="F11" t="n">
-        <v>18.9</v>
+        <v>18.88</v>
       </c>
       <c r="G11" t="n">
-        <v>73.3</v>
+        <v>73.34</v>
       </c>
     </row>
     <row r="12">
@@ -915,7 +915,7 @@
         <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G12" t="n">
         <v>100</v>
@@ -939,13 +939,13 @@
         <v>9</v>
       </c>
       <c r="E13" t="n">
-        <v>22.2</v>
+        <v>22.22</v>
       </c>
       <c r="F13" t="n">
-        <v>6.3</v>
+        <v>6.32</v>
       </c>
       <c r="G13" t="n">
-        <v>54.7</v>
+        <v>54.74</v>
       </c>
     </row>
     <row r="14">
@@ -969,7 +969,7 @@
         <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G14" t="n">
         <v>100</v>
@@ -996,7 +996,7 @@
         <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G15" t="n">
         <v>100</v>
@@ -1023,7 +1023,7 @@
         <v>100</v>
       </c>
       <c r="F16" t="n">
-        <v>70.09999999999999</v>
+        <v>70.08</v>
       </c>
       <c r="G16" t="n">
         <v>100</v>
@@ -1047,13 +1047,13 @@
         <v>9</v>
       </c>
       <c r="E17" t="n">
-        <v>88.90000000000001</v>
+        <v>88.89</v>
       </c>
       <c r="F17" t="n">
         <v>56.5</v>
       </c>
       <c r="G17" t="n">
-        <v>98</v>
+        <v>98.01000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>